<commit_message>
Site guncellemesi - 14.09.2026 18:32
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,136 +35,97 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>ALARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBRK</x:t>
-  </x:si>
-  <x:si>
     <x:t>ALKLC</x:t>
   </x:si>
   <x:si>
-    <x:t>AVGYO</x:t>
-  </x:si>
-  <x:si>
     <x:t>AVPGY</x:t>
   </x:si>
   <x:si>
     <x:t>BAHKM</x:t>
   </x:si>
   <x:si>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETILR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUKYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSDDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HURGZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IEYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KCHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSYN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRCAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANHYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYGAZ</x:t>
+  </x:si>
+  <x:si>
     <x:t>BIMAS</x:t>
   </x:si>
   <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EBEBK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGPRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENJSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUKYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HURGZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IEYHO</x:t>
+    <x:t>CATES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOHOL</x:t>
   </x:si>
   <x:si>
     <x:t>ISDMR</x:t>
   </x:si>
   <x:si>
-    <x:t>KCHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRPLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRALT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRCAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ADGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYDEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CATES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HALKB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KERVN</x:t>
-  </x:si>
-  <x:si>
     <x:t>METRO</x:t>
   </x:si>
   <x:si>
-    <x:t>PETKM</x:t>
+    <x:t>NETAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZATD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RALYH</x:t>
   </x:si>
   <x:si>
     <x:t>SKYMD</x:t>
@@ -174,12 +135,6 @@
   </x:si>
   <x:si>
     <x:t>TNZTP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRENJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRMET</x:t>
   </x:si>
   <x:si>
     <x:t>TUPRS</x:t>
@@ -533,7 +488,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C32"/>
+  <x:dimension ref="A1:C21"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -764,127 +719,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" spans="1:3">
-      <x:c r="A22" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C22" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" spans="1:3">
-      <x:c r="A23" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C23" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" spans="1:3">
-      <x:c r="A24" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C24" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" spans="1:3">
-      <x:c r="A25" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C25" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" spans="1:3">
-      <x:c r="A26" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C26" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" spans="1:3">
-      <x:c r="A27" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B27" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C27" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" spans="1:3">
-      <x:c r="A28" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B28" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C28" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" spans="1:3">
-      <x:c r="A29" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B29" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C29" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" spans="1:3">
-      <x:c r="A30" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B30" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C30" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" spans="1:3">
-      <x:c r="A31" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B31" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C31" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" spans="1:3">
-      <x:c r="A32" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B32" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C32" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -902,7 +736,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C21"/>
+  <x:dimension ref="A1:C17"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -918,7 +752,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -929,7 +763,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -940,7 +774,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -951,7 +785,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -962,7 +796,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -973,7 +807,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -984,7 +818,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -995,7 +829,7 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
@@ -1006,7 +840,7 @@
     </x:row>
     <x:row r="10" spans="1:3">
       <x:c r="A10" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
         <x:v>4</x:v>
@@ -1017,7 +851,7 @@
     </x:row>
     <x:row r="11" spans="1:3">
       <x:c r="A11" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
         <x:v>4</x:v>
@@ -1028,7 +862,7 @@
     </x:row>
     <x:row r="12" spans="1:3">
       <x:c r="A12" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
         <x:v>4</x:v>
@@ -1039,7 +873,7 @@
     </x:row>
     <x:row r="13" spans="1:3">
       <x:c r="A13" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>4</x:v>
@@ -1050,7 +884,7 @@
     </x:row>
     <x:row r="14" spans="1:3">
       <x:c r="A14" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>4</x:v>
@@ -1061,7 +895,7 @@
     </x:row>
     <x:row r="15" spans="1:3">
       <x:c r="A15" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>4</x:v>
@@ -1072,7 +906,7 @@
     </x:row>
     <x:row r="16" spans="1:3">
       <x:c r="A16" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>4</x:v>
@@ -1083,56 +917,12 @@
     </x:row>
     <x:row r="17" spans="1:3">
       <x:c r="A17" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" spans="1:3">
-      <x:c r="A18" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C18" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:3">
-      <x:c r="A19" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C19" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:3">
-      <x:c r="A20" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C20" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" spans="1:3">
-      <x:c r="A21" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C21" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 15.09.2026 18:34
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -41,100 +41,49 @@
     <x:t>AVPGY</x:t>
   </x:si>
   <x:si>
-    <x:t>BAHKM</x:t>
+    <x:t>BMSTL</x:t>
   </x:si>
   <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
+    <x:t>DSTKF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EFOR</x:t>
   </x:si>
   <x:si>
     <x:t>ENERY</x:t>
   </x:si>
   <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
     <x:t>EUKYO</x:t>
   </x:si>
   <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HURGZ</x:t>
-  </x:si>
-  <x:si>
     <x:t>IEYHO</x:t>
   </x:si>
   <x:si>
-    <x:t>KCHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKM</x:t>
-  </x:si>
-  <x:si>
     <x:t>TEHOL</x:t>
   </x:si>
   <x:si>
-    <x:t>TRCAS</x:t>
+    <x:t>TNZTP</x:t>
   </x:si>
   <x:si>
     <x:t>TRHOL</x:t>
   </x:si>
   <x:si>
-    <x:t>AGHOL</x:t>
-  </x:si>
-  <x:si>
     <x:t>ANHYT</x:t>
   </x:si>
   <x:si>
-    <x:t>ARSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CATES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOHOL</x:t>
-  </x:si>
-  <x:si>
     <x:t>ISDMR</x:t>
   </x:si>
   <x:si>
-    <x:t>METRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NETAS</x:t>
-  </x:si>
-  <x:si>
     <x:t>OZATD</x:t>
   </x:si>
   <x:si>
-    <x:t>RALYH</x:t>
-  </x:si>
-  <x:si>
     <x:t>SKYMD</x:t>
   </x:si>
   <x:si>
     <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TNZTP</x:t>
   </x:si>
   <x:si>
     <x:t>TUPRS</x:t>
@@ -488,7 +437,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C21"/>
+  <x:dimension ref="A1:C14"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -642,83 +591,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:3">
-      <x:c r="A15" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C15" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" spans="1:3">
-      <x:c r="A16" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C16" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:3">
-      <x:c r="A17" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C17" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" spans="1:3">
-      <x:c r="A18" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C18" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:3">
-      <x:c r="A19" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C19" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:3">
-      <x:c r="A20" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C20" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" spans="1:3">
-      <x:c r="A21" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C21" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -736,7 +608,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C17"/>
+  <x:dimension ref="A1:C7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -752,7 +624,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -763,7 +635,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -774,7 +646,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -785,7 +657,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -796,7 +668,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -807,122 +679,12 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:3">
-      <x:c r="A9" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:3">
-      <x:c r="A10" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:3">
-      <x:c r="A11" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:3">
-      <x:c r="A12" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:3">
-      <x:c r="A13" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C13" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:3">
-      <x:c r="A14" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C14" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:3">
-      <x:c r="A15" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C15" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" spans="1:3">
-      <x:c r="A16" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C16" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:3">
-      <x:c r="A17" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C17" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 16.09.2026 18:30
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,7 +26,7 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>AHGAZ</x:t>
+    <x:t>BMSTL</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
@@ -35,58 +35,16 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>ALKLC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVPGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BMSTL</x:t>
+    <x:t>EFOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUKYO</x:t>
   </x:si>
   <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
-    <x:t>DSTKF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EFOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUKYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IEYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TNZTP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANHYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZATD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
     <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUPRS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -437,7 +395,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C14"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -481,116 +439,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:3">
-      <x:c r="A9" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:3">
-      <x:c r="A10" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:3">
-      <x:c r="A11" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:3">
-      <x:c r="A12" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:3">
-      <x:c r="A13" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C13" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:3">
-      <x:c r="A14" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C14" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -608,7 +456,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C7"/>
+  <x:dimension ref="A1:C3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -624,7 +472,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -635,56 +483,12 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 18.09.2026 18:38
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,46 +26,37 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAHKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EFOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISDMR</x:t>
+  </x:si>
+  <x:si>
     <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANHYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BMSTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HALKB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
   </x:si>
   <x:si>
     <x:t>TUPRS</x:t>
@@ -419,7 +410,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C2"/>
+  <x:dimension ref="A1:C1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -431,17 +422,6 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
-      <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -458,7 +438,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C13"/>
+  <x:dimension ref="A1:C11"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -474,7 +454,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -485,7 +465,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -496,7 +476,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -507,7 +487,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -518,7 +498,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -529,7 +509,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -540,7 +520,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -551,7 +531,7 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
@@ -562,7 +542,7 @@
     </x:row>
     <x:row r="10" spans="1:3">
       <x:c r="A10" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
         <x:v>4</x:v>
@@ -573,34 +553,12 @@
     </x:row>
     <x:row r="11" spans="1:3">
       <x:c r="A11" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:3">
-      <x:c r="A12" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:3">
-      <x:c r="A13" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C13" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 21.09.2026 18:38
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,34 +26,31 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>BAHKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
     <x:t>AHGAZ</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAHKM</x:t>
-  </x:si>
-  <x:si>
     <x:t>BIMAS</x:t>
   </x:si>
   <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EFOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INVES</x:t>
-  </x:si>
-  <x:si>
     <x:t>ISDMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KCHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKM</x:t>
   </x:si>
   <x:si>
     <x:t>TKFEN</x:t>
@@ -410,7 +407,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C1"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -422,6 +419,17 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -438,7 +446,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C11"/>
+  <x:dimension ref="A1:C9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -454,7 +462,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -465,7 +473,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -476,7 +484,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -487,7 +495,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -498,7 +506,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -509,7 +517,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -520,7 +528,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -531,34 +539,12 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:3">
-      <x:c r="A10" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:3">
-      <x:c r="A11" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 22.09.2026 18:39
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,37 +26,46 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
     <x:t>BAHKM</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
     <x:t>BIMAS</x:t>
   </x:si>
   <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
     <x:t>ISDMR</x:t>
   </x:si>
   <x:si>
     <x:t>KCHOL</x:t>
   </x:si>
   <x:si>
+    <x:t>KRDMD</x:t>
+  </x:si>
+  <x:si>
     <x:t>RYGYO</x:t>
   </x:si>
   <x:si>
-    <x:t>SOKM</x:t>
-  </x:si>
-  <x:si>
     <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUPRS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -407,7 +416,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C2"/>
+  <x:dimension ref="A1:C5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -429,6 +438,39 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -462,7 +504,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -473,7 +515,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -484,7 +526,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -495,7 +537,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -506,7 +548,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -517,7 +559,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -528,7 +570,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -539,7 +581,7 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>

</xml_diff>

<commit_message>
Site guncellemesi - 29.09.2026 18:58
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,37 +35,25 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FLAP</x:t>
+  </x:si>
+  <x:si>
     <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAHKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FLAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -416,7 +404,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C7"/>
+  <x:dimension ref="A1:C6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -482,17 +470,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -510,7 +487,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C7"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -526,7 +503,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -537,7 +514,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -548,45 +525,12 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 30.09.2026 18:31
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -38,22 +38,19 @@
     <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
+    <x:t>SKYMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
     <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FLAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -404,7 +401,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -448,28 +445,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -487,7 +462,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -503,7 +478,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -514,7 +489,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -525,12 +500,23 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 01.10.2026 18:26
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,31 +26,40 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
     <x:t>ETILR</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
     <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
     <x:t>SKYMD</x:t>
   </x:si>
   <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FLAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKFEN</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -401,7 +410,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -445,6 +454,50 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:3">
+      <x:c r="A6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:3">
+      <x:c r="A8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -462,7 +515,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C5"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -478,7 +531,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -489,7 +542,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -500,23 +553,12 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 02.10.2026 18:31
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,6 +35,9 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
+    <x:t>AKFIS</x:t>
+  </x:si>
+  <x:si>
     <x:t>ENERY</x:t>
   </x:si>
   <x:si>
@@ -47,19 +50,13 @@
     <x:t>HRKET</x:t>
   </x:si>
   <x:si>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
     <x:t>HUNER</x:t>
   </x:si>
   <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FLAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
+    <x:t>KRPLS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -410,7 +407,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C8"/>
+  <x:dimension ref="A1:C7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -487,17 +484,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -531,7 +517,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -542,7 +528,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -553,7 +539,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>

</xml_diff>

<commit_message>
Site guncellemesi - 06.10.2026 18:33
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,25 +35,28 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>AKFIS</x:t>
+    <x:t>AVGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRSAN</x:t>
   </x:si>
   <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
     <x:t>ENERY</x:t>
   </x:si>
   <x:si>
-    <x:t>ETILR</x:t>
+    <x:t>INDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYGYO</x:t>
   </x:si>
   <x:si>
     <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
   </x:si>
   <x:si>
     <x:t>TKFEN</x:t>
@@ -407,7 +410,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C5"/>
+  <x:dimension ref="A1:C9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -462,6 +465,50 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:3">
+      <x:c r="A6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:3">
+      <x:c r="A8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:3">
+      <x:c r="A9" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -479,7 +526,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -495,7 +542,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -506,45 +553,12 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 08.10.2026 18:36
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -38,9 +38,6 @@
     <x:t>ALBRK</x:t>
   </x:si>
   <x:si>
-    <x:t>AVGYO</x:t>
-  </x:si>
-  <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
@@ -50,16 +47,13 @@
     <x:t>ENERY</x:t>
   </x:si>
   <x:si>
+    <x:t>ENJSA</x:t>
+  </x:si>
+  <x:si>
     <x:t>HRKET</x:t>
   </x:si>
   <x:si>
-    <x:t>AKFIS</x:t>
-  </x:si>
-  <x:si>
     <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -515,7 +509,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -537,28 +531,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 12.10.2026 18:24
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,46 +35,28 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>AKFIS</x:t>
-  </x:si>
-  <x:si>
     <x:t>ALBRK</x:t>
   </x:si>
   <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORGE</x:t>
+  </x:si>
+  <x:si>
     <x:t>CELHA</x:t>
   </x:si>
   <x:si>
     <x:t>DURDO</x:t>
   </x:si>
   <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENJSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
     <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
   </x:si>
   <x:si>
     <x:t>VAKBN</x:t>
@@ -428,7 +410,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C10"/>
+  <x:dimension ref="A1:C7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -505,39 +487,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:3">
-      <x:c r="A9" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:3">
-      <x:c r="A10" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -555,7 +504,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C8"/>
+  <x:dimension ref="A1:C5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -571,7 +520,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -582,7 +531,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -593,7 +542,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -604,45 +553,12 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 14.10.2026 18:25
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,7 +26,7 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>ENERY</x:t>
+    <x:t>DURDO</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
@@ -35,28 +35,31 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>ENJSA</x:t>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKBN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKFIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALARK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
   </x:si>
   <x:si>
     <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
   </x:si>
   <x:si>
     <x:t>RYGYO</x:t>
@@ -493,7 +496,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -559,6 +562,17 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 15.10.2026 18:34
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,7 +26,7 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>DURDO</x:t>
+    <x:t>ENJSA</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
@@ -38,31 +38,22 @@
     <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
     <x:t>INDES</x:t>
   </x:si>
   <x:si>
     <x:t>SOKM</x:t>
   </x:si>
   <x:si>
-    <x:t>VAKBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFIS</x:t>
+    <x:t>AHGAZ</x:t>
   </x:si>
   <x:si>
     <x:t>ALARK</x:t>
   </x:si>
   <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
+    <x:t>ENERY</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -496,7 +487,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C7"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -540,39 +531,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 16.10.2026 18:37
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,7 +26,7 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>ENJSA</x:t>
+    <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
@@ -35,25 +35,10 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
+    <x:t>RYSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -404,7 +389,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C6"/>
+  <x:dimension ref="A1:C3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -437,39 +422,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -487,7 +439,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -503,34 +455,12 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 19.10.2026 19:44
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,10 +35,7 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>RYSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLYHO</x:t>
+    <x:t>SOKM</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -439,7 +436,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C2"/>
+  <x:dimension ref="A1:C1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -451,17 +448,6 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
-      <x:c r="A2" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Site guncellemesi - 20.10.2026 18:50
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,13 +26,34 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>ENJSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
     <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETILR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INDES</x:t>
   </x:si>
   <x:si>
     <x:t>SOKM</x:t>
@@ -436,7 +457,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C1"/>
+  <x:dimension ref="A1:C8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -448,6 +469,83 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:3">
+      <x:c r="A6" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:3">
+      <x:c r="A8" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Site guncellemesi - 21.10.2026 18:43
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -35,28 +35,10 @@
     <x:t>TL</x:t>
   </x:si>
   <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
     <x:t>ETILR</x:t>
   </x:si>
   <x:si>
-    <x:t>GLYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKM</x:t>
+    <x:t>RYGYO</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -407,7 +389,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C3"/>
+  <x:dimension ref="A1:C1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -419,28 +401,6 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
-      <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -457,7 +417,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C8"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -473,7 +433,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -484,7 +444,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -495,56 +455,12 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
-      <x:c r="A5" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
-      <x:c r="A6" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 23.10.2026 10:34
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,19 +26,13 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>ENJSA</x:t>
+    <x:t>RYGYO</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
   </x:si>
   <x:si>
     <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -417,7 +411,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -439,28 +433,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 23.10.2026 19:40
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,13 +26,25 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>DOCO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSYN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
     <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -383,7 +395,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C1"/>
+  <x:dimension ref="A1:C3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -395,6 +407,28 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -411,7 +445,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C2"/>
+  <x:dimension ref="A1:C4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -427,12 +461,34 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Site guncellemesi - 27.10.2026 18:52
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,22 +26,13 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
-    <x:t>DOCO</x:t>
+    <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
     <x:t>Gün</x:t>
   </x:si>
   <x:si>
     <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
     <x:t>RYGYO</x:t>
@@ -445,7 +436,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -457,39 +448,6 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
-      <x:c r="A2" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
-      <x:c r="A3" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
-      <x:c r="A4" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Site guncellemesi - 30.10.2026 19:32
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
+++ b/app/borsa/gosterge-taramalari/data/guclu-trend-momentum.xlsx
@@ -26,16 +26,19 @@
     <x:t>Birim</x:t>
   </x:si>
   <x:si>
+    <x:t>DOCO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gün</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TL</x:t>
+  </x:si>
+  <x:si>
     <x:t>GMTAS</x:t>
   </x:si>
   <x:si>
-    <x:t>Gün</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
+    <x:t>AHGAZ</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -436,7 +439,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C1"/>
+  <x:dimension ref="A1:C2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -448,6 +451,17 @@
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>